<commit_message>
feat: dataset test openai
</commit_message>
<xml_diff>
--- a/nbd_backend/evaluation/metrics_output/evaluation_report.xlsx
+++ b/nbd_backend/evaluation/metrics_output/evaluation_report.xlsx
@@ -63,12 +63,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -112,39 +112,39 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -512,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -585,23 +585,23 @@
       <c r="C2" s="4" t="n">
         <v>0.5161</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>0.6696</v>
-      </c>
-      <c r="E2" s="5" t="n">
+      <c r="D2" s="5" t="n">
+        <v>0.1667</v>
+      </c>
+      <c r="E2" s="6" t="n">
         <v>0.7961</v>
       </c>
-      <c r="F2" s="4" t="n">
-        <v>0.7234</v>
+      <c r="F2" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>heuristic_fallback</t>
+          <t>ragas</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>heuristic_fallback</t>
+          <t>ragas</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
@@ -609,317 +609,37 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Tại sao bệnh nhân hít thở FiO2 cao (nồng độ oxy cao) lại có nguy cơ tiến triển xẹp phổi tái hấp thu nhanh hơn?</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="5" t="n">
         <v>0.4074</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>0.514</v>
+      <c r="D3" s="5" t="n">
+        <v>0.3333</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0.723</v>
       </c>
-      <c r="F3" s="4" t="n">
-        <v>0.5111</v>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="b">
+      <c r="F3" s="5" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" ht="45" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Dấu hiệu 'Golden S sign' (dấu hiệu S ngược) trên X-quang thường gợi ý bệnh lý gì và tại sao?</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>0.3498</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>0.3636</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0.6454</v>
-      </c>
-      <c r="F4" s="8" t="n">
-        <v>0.4151</v>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Dấu hiệu 'Luftsichel sign' là gì và nó giúp chẩn đoán tình trạng nào?</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>0.3109</v>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>0.4444</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>0.6408</v>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>0.2632</v>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Tại sao trong xẹp phổi, trung thất và khí quản lại bị lệch về phía tổn thương?</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0.5327</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>0.7917</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>0.7682</v>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>0.4878</v>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Dấu hiệu 'Retrocardiac sail sign' (cánh buồm sau tim) có ý nghĩa gì trong chẩn đoán hình ảnh?</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>0.2618</v>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>0.3214</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>0.6734</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>0.3571</v>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Sự khác biệt về rung thanh (vocal fremitus) giữa xẹp phổi và đông đặc phổi là gì?</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>0.4262</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>0.625</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>0.7034</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0.6667</v>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Cơ chế 'Xẹp phổi do kết dính' (Adhesive Atelectasis) có liên quan đến thành phần nào trong phế nang?</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>0.6102</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>0.5088</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>0.6655</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0.5946</v>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Tại sao rốn phổi phải có thể bị kéo giật lên cao trong xẹp thùy trên phải?</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>0.4957</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>0.7681</v>
-      </c>
-      <c r="F10" s="8" t="n">
-        <v>0.3488</v>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Nêu tiêu chí chẩn đoán phân biệt chính giữa xẹp phổi tắc nghẽn và tràn dịch màng phổi lượng lớn dựa trên sự di lệch trung thất.</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>0.5271</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>0.6353</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="F11" s="8" t="n">
-        <v>0.4103</v>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>heuristic_fallback</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="b">
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>ragas</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>ragas</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -978,16 +698,16 @@
         </is>
       </c>
       <c r="B2" s="11" t="n">
-        <v>0.4438</v>
+        <v>0.4617</v>
       </c>
       <c r="C2" s="12" t="n">
-        <v>0.1057</v>
+        <v>0.0544</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>0.2618</v>
+        <v>0.4074</v>
       </c>
       <c r="E2" s="12" t="n">
-        <v>0.6102</v>
+        <v>0.5161</v>
       </c>
     </row>
     <row r="3">
@@ -996,17 +716,17 @@
           <t>Faithfulness</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
-        <v>0.5514</v>
+      <c r="B3" s="11" t="n">
+        <v>0.25</v>
       </c>
       <c r="C3" s="12" t="n">
-        <v>0.1396</v>
+        <v>0.0833</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>0.3214</v>
+        <v>0.1667</v>
       </c>
       <c r="E3" s="12" t="n">
-        <v>0.7917</v>
+        <v>0.3333</v>
       </c>
     </row>
     <row r="4">
@@ -1016,13 +736,13 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>0.706</v>
+        <v>0.7595</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>0.0526</v>
+        <v>0.0366</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>0.6408</v>
+        <v>0.723</v>
       </c>
       <c r="E4" s="12" t="n">
         <v>0.7961</v>
@@ -1035,16 +755,16 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>0.4778</v>
+        <v>0</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>0.1402</v>
+        <v>0</v>
       </c>
       <c r="D5" s="12" t="n">
-        <v>0.2632</v>
+        <v>0</v>
       </c>
       <c r="E5" s="12" t="n">
-        <v>0.7234</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1054,7 +774,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">

</xml_diff>